<commit_message>
Billing App v4.0 - Finance tracker, Edit/Delete, Course Plans
</commit_message>
<xml_diff>
--- a/robokidy_billing_data.xlsx
+++ b/robokidy_billing_data.xlsx
@@ -11,7 +11,9 @@
     <sheet name="Students" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Invoices" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Payments" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Settings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CoursePlans" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Finance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Settings" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -449,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -471,7 +473,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>03-06-2026 10:36 AM</t>
+          <t>04-06-2026 09:56 AM</t>
         </is>
       </c>
     </row>
@@ -482,7 +484,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -492,7 +494,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -502,7 +504,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -512,7 +514,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-63000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -522,7 +524,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -532,7 +534,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-70000</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Total Income</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Total Expenses</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Net Profit</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -546,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -637,73 +669,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>RK-SC-L2-2026-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>NIVIIN</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>BALA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>12433</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>BALA</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Scratch</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Afternoon</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>03-06-2026</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>22222</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -715,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -848,87 +813,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>RKI-INV-2026-0001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>03-06-2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>RK-SC-L2-2026-001</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>NIVIIN</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Scratch</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Afternoon</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>7000</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="K2" t="n">
-        <v>70000</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>-63000</v>
-      </c>
-      <c r="P2" t="n">
-        <v>7000</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>-70000</v>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Cash</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -940,7 +824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1001,57 +885,494 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>RKI-RCP-2026-0001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>03-06-2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>RKI-INV-2026-0001</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>RK-SC-L2-2026-001</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>NIVIIN</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>7000</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Initial payment</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Plan ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Fee</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PLN-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Level 1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Python basics</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PLN-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Level 2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Python advanced</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PLN-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Robotics</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Level 1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Robotics basics</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PLN-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Arduino</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Level 1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Arduino basics</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PLN-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Scratch</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Level 1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Scratch basics</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PLN-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AI/ML</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Level 1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>AI/ML monthly</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PLN-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IoT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Level 1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>IoT monthly</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PLN-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Web Dev</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Level 1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Web Dev monthly</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PLN-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Yearly All-Courses</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>All Levels</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Yearly</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>25000</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>All courses yearly plan</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PLN-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Yearly All-Courses</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>All Levels</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Half-Yearly</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>14000</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>All courses half-yearly</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Entry ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Payment Mode</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>